<commit_message>
data: operator added 3 orphan ASINs to master + ETL refresh
Operator added B0G1YKMFWT (Nexlev, W16 sales) and B0GYS6CJD9 (Nexlev,
W20+W21 sales) to sku_master.  Also looks like B0DS2HLR6S (White
Mulberry, W16 sessions-only) was added.

Sync resolved 4 raw cells via direct ASIN lookup now (no longer via
SKU fallback).  Orphan count dropped from 6 unique → 3 — only the
zero-sales Audio Array session-only listings remain (B0FR8XJFJ3,
B0GWPYFLWG, B0GWQ4T8MV in W17), which the operator chose to ignore
per the triage call.

ETL chain re-run; ams_weekly_fact, business_ads_joined, weekly_sales
and inbound snapshots regenerated.  Sales for the now-resolved ASINs
attribute correctly to their canonical models.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Nexlev/business_report_week20.xlsx
+++ b/data/ams_weekly_data/Nexlev/business_report_week20.xlsx
@@ -3905,6 +3905,16 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FBA80113</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SC-01_Mop_Cloth</t>
+        </is>
+      </c>
       <c r="C43" t="inlineStr">
         <is>
           <t>B0GYS6CJD9</t>

</xml_diff>